<commit_message>
test: +14 tests manquants ajoutés au fichier consolidé (297 total)
Ajouts par onglet:
- Projets (+9): E-14 services transversaux, E-35 11 colonnes,
  E-25 label Factures, E-29 bouton Paramètres, E-38 colonne Projet,
  E-19 sous-tâches, E-39/40 transfert responsable,
  consortium membres + coefficients, consortium vue duale FR61
- Auth & Navigation (+2): ECART-SECU-01 employé /billing,
  employé /consortiums bloqué
- Dashboard & Admin (+3): E-05 liste projets dashboard,
  E-08 bienvenue prénom, E-04 4 KPIs PM

Couverture: 38/38 features vérifiées ✅

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests_consolides_par_module.xlsx
+++ b/backend/tests_consolides_par_module.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1408,6 +1408,85 @@
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
     </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>SEC-B2-01</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité accès</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Employé ne peut pas accéder à /billing</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Employé</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Connexion employé (pas PM/Finance)</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>1. Se connecter comme employe@test.com
+2. Naviguer vers /billing</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Redirection automatique vers /dashboard (route guard)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>SEC-B2-02</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Sécurité accès</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Employé ne peut pas accéder à /consortiums</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>Employé</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Connexion employé</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>1. Naviguer vers /consortiums</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Redirection vers /dashboard</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1419,7 +1498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2700,6 +2779,127 @@
         </is>
       </c>
       <c r="I32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>DASH-NEW-01</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard PM</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Liste projets visible dans le dashboard (E-05)</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Projets actifs assignés</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>1. /dashboard
+2. Section "Chef de projet"
+3. Vérifier table projets</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Table avec Code, Projet, Client, Phase active, Budget h, Santé + lien "Voir tous les projets"</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n"/>
+      <c r="I33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>DASH-NEW-02</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard PM</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Message bienvenue avec prénom (E-08)</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Connexion</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>1. /dashboard
+2. Vérifier header</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>"Bienvenue, [Prénom]" + date du jour en français</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n"/>
+      <c r="I34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>DASH-NEW-03</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard PM</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>4 KPIs PM (E-04)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Projets avec données</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>1. /dashboard section PM
+2. Vérifier 4 KPIs</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Heures ce mois, Ratio CA/Salaires (cible 2.5x), Taux facturation, Actions requises</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n"/>
+      <c r="I35" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3229,7 +3429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6304,6 +6504,378 @@
       </c>
       <c r="H79" s="4" t="n"/>
       <c r="I79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>P-108</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Services transversaux (E-14)</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Sélectionner services transversaux dans wizard</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Wizard étape 1</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>1. Ouvrir wizard
+2. Cliquer sur BIM, DD, Paysage
+3. Vérifier toggle actif/inactif
+4. Créer le projet</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Services enregistrés (services_transversaux=["BIM","DD","PAYSAGE"]) et affichés dans Vue d'ensemble</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>P-109</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Colonnes liste (E-35)</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier 11 colonnes dans la liste projets</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Plusieurs projets</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>1. /projects
+2. Vérifier colonnes: Code, Projet, Client, Chef de projet, BU, Phase active, Budget h, CA, Statut, Santé</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>11 colonnes affichées avec données correctes</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="n"/>
+      <c r="I81" s="4" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>P-110</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Label Factures (E-25)</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier onglet "Factures" (pas "Facturation")</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Projet existant</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet
+2. Vérifier nom du dernier onglet</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>Onglet nommé "Factures" (pas "Facturation")</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>P-111</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Bouton Paramètres (E-29)</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier bouton "⚙️ Paramètres" (pas "Modifier")</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Projet existant</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet
+2. Vérifier bouton en haut à droite</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Bouton "⚙️ Paramètres" visible (pas "Modifier")</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>P-112</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Colonne Projet (E-38)</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier colonne "Projet" (pas "Nom") dans la liste</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Liste projets</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>1. /projects
+2. Vérifier le header de la 2e colonne</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>Colonne nommée "Projet" (pas "Nom")</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>P-113</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Sous-tâches (E-19)</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Créer une sous-tâche dans l'onglet Tâches</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Projet avec tâches, mode édition</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>1. Ouvrir fiche projet &gt; Tâches
+2. Cliquer ⚙️ Paramètres
+3. Cliquer "+ ST" sur une tâche
+4. Saisir nom
+5. Valider</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>Sous-tâche créée avec task_type=SUBTASK, WBS code parent.N, indentation visible</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>P-114</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Transfert responsable (E-39/E-40)</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Transférer le PM d'un projet</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>ADMIN</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Projet avec PM assigné</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>1. /projects/transfer
+2. Sélectionner projet
+3. Type: Chef de projet
+4. Sélectionner nouveau PM
+5. Valider</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>PM mis à jour, historique affiché, ancien PM visible</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="n"/>
+      <c r="I86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>P-115</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Consortium membres</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Ajouter membres avec coefficients dans le formulaire</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Consortium créé</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>1. /consortiums/{id}/edit
+2. Vérifier PR auto-ajouté
+3. Cliquer "+ Ajouter partenaire"
+4. Sélectionner org, coefficient 60%
+5. Vérifier NEQ affiché
+6. Vérifier total = 100%</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>PR (40%) + partenaire (60%) = 100%, NEQ visible, lien "Voir fiche"</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>P-116</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Consortium vue duale (FR61)</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Vérifier les 6 onglets du consortium</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Consortium avec membres + projet lié</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>1. /consortiums/{id}
+2. Parcourir les 6 onglets: Vue d'ensemble, Vue duale, Projets, Factures partenaires, Distributions, Déclarations taxes</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>Vue duale: panneau bleu (consortium) + panneau jaune (Provencher), tableau comparatif 3 modes</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>